<commit_message>
Make hourly scheduling resilient and skip duplicate 6174 topic
</commit_message>
<xml_diff>
--- a/input/prompts.xlsx
+++ b/input/prompts.xlsx
@@ -527,7 +527,6 @@
           <t>2026-09-13T18:25:45.481701+00:00</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="11" t="inlineStr">
@@ -970,7 +969,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>SKIPPED_DUPLICATE</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Duplicate topic: Kaprekar constant 6174 is already uploaded as prompt 31.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix cross-topic review contamination and rate-limit handling
</commit_message>
<xml_diff>
--- a/input/prompts.xlsx
+++ b/input/prompts.xlsx
@@ -459,12 +459,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Content quality review failed: Incorrect count of four‑digit strings (should be 10000, not 9000).; Wrong worst‑case iteration claim for 1098 (it reaches 6174 in 3 steps, not 7).</t>
+          <t>PENDING</t>
         </is>
       </c>
     </row>
@@ -479,12 +474,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Error code: 413 - {'error': {'message': 'Request too large for model `openai/gpt-oss-120b` in organization `org_01kzfy82cxeyvbp25hn08bgge3` service tier `on_demand` on tokens per minute (TPM): Limit 8000, Requested 9270, please reduce your message size and try again. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'tokens', 'code': 'rate_limit_exceeded'}}</t>
+          <t>PENDING</t>
         </is>
       </c>
     </row>
@@ -539,14 +529,10 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Content quality review failed: Incorrect claim that the Kaprekar constant appears in "base‑110"; the discussion should be limited to base‑10 only.</t>
-        </is>
-      </c>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7" ht="34" customHeight="1">
       <c r="A7" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Restore prompts affected by exhausted quota
</commit_message>
<xml_diff>
--- a/input/prompts.xlsx
+++ b/input/prompts.xlsx
@@ -459,12 +459,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Error code: 429 - {'error': {'message': 'Rate limit reached for model `openai/gpt-oss-120b` in organization `org_01kzfy82cxeyvbp25hn08bgge3` service tier `on_demand` on tokens per day (TPD): Limit 200000, Used 199849, Requested 3462. Please try again in 23m50.352s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'tokens', 'code': 'rate_limit_exceeded'}}</t>
+          <t>PENDING</t>
         </is>
       </c>
     </row>
@@ -479,14 +474,10 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Error code: 429 - {'error': {'message': 'Rate limit reached for model `openai/gpt-oss-120b` in organization `org_01kzfy82cxeyvbp25hn08bgge3` service tier `on_demand` on tokens per day (TPD): Limit 200000, Used 199849, Requested 1177. Please try again in 7m23.232s. Need more tokens? Upgrade to Dev Tier today at https://console.groq.com/settings/billing', 'type': 'tokens', 'code': 'rate_limit_exceeded'}}</t>
-        </is>
-      </c>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Restore prompt after JSON formatting failure
</commit_message>
<xml_diff>
--- a/input/prompts.xlsx
+++ b/input/prompts.xlsx
@@ -459,14 +459,10 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FAILED</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Invalid \escape: line 1 column 628 (char 627)</t>
-        </is>
-      </c>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4" ht="34" customHeight="1">
       <c r="A4" s="11" t="inlineStr">
@@ -507,7 +503,6 @@
           <t>2026-09-13T22:37:26.191669+00:00</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="11" t="inlineStr">

</xml_diff>